<commit_message>
Extraccion de datos de Italia, datos missing y reentrenamiento de modelos
</commit_message>
<xml_diff>
--- a/p3_data_preparation/data/italy/clean_data/df_teams_sofifa_cleaned.xlsx
+++ b/p3_data_preparation/data/italy/clean_data/df_teams_sofifa_cleaned.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:I41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -694,35 +694,35 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>110374</v>
+        <v>39</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>fiorentina</t>
+          <t>atalanta</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Stadio Classico</t>
+          <t>Home stadium</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E8" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F8" t="n">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Juventus</t>
+          <t>Milan</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>https://sofifa.com/team/110374/fiorentina/</t>
+          <t>https://sofifa.com/team/39/atalanta/</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -731,35 +731,35 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>39</v>
+        <v>110374</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>atalanta</t>
+          <t>fiorentina</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Home stadium</t>
+          <t>Stadio Classico</t>
         </is>
       </c>
       <c r="D9" t="n">
+        <v>5</v>
+      </c>
+      <c r="E9" t="n">
         <v>6</v>
       </c>
-      <c r="E9" t="n">
-        <v>7</v>
-      </c>
       <c r="F9" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Milan</t>
+          <t>Juventus</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://sofifa.com/team/39/atalanta/</t>
+          <t>https://sofifa.com/team/110374/fiorentina/</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -805,35 +805,35 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>111974</v>
+        <v>189</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>sassuolo</t>
+          <t>bologna</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Forest Park Stadium (Square Ground)</t>
+          <t>Euro Arena</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E11" t="n">
         <v>4</v>
       </c>
       <c r="F11" t="n">
-        <v>189</v>
+        <v>110374</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Bologna</t>
+          <t>Fiorentina</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://sofifa.com/team/111974/sassuolo/</t>
+          <t>https://sofifa.com/team/189/bologna/</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -842,35 +842,35 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>189</v>
+        <v>111974</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>bologna</t>
+          <t>sassuolo</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Euro Arena</t>
+          <t>Forest Park Stadium (Square Ground)</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E12" t="n">
         <v>4</v>
       </c>
       <c r="F12" t="n">
-        <v>110374</v>
+        <v>189</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Fiorentina</t>
+          <t>Bologna</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>https://sofifa.com/team/189/bologna/</t>
+          <t>https://sofifa.com/team/111974/sassuolo/</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -990,35 +990,35 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>1746</v>
+        <v>110556</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>empoli</t>
+          <t>genoa</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Euro Arena</t>
+          <t>Stadion Europa</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E16" t="n">
         <v>2</v>
       </c>
       <c r="F16" t="n">
-        <v>110374</v>
+        <v>1837</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Fiorentina</t>
+          <t>Sampdoria</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>https://sofifa.com/team/1746/empoli/</t>
+          <t>https://sofifa.com/team/110556/genoa/</t>
         </is>
       </c>
       <c r="I16" t="n">
@@ -1027,35 +1027,35 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>110556</v>
+        <v>1842</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>genoa</t>
+          <t>cagliari</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Stadion Europa</t>
+          <t>Stadio Classico</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E17" t="n">
         <v>2</v>
       </c>
       <c r="F17" t="n">
-        <v>1837</v>
+        <v>48</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Sampdoria</t>
+          <t>Napoli</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://sofifa.com/team/110556/genoa/</t>
+          <t>https://sofifa.com/team/1842/cagliari/</t>
         </is>
       </c>
       <c r="I17" t="n">
@@ -1064,23 +1064,23 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>1842</v>
+        <v>206</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>cagliari</t>
+          <t>hellas verona</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Stadio Classico</t>
+          <t>Sanderson Park</t>
         </is>
       </c>
       <c r="D18" t="n">
         <v>1</v>
       </c>
       <c r="E18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F18" t="n">
         <v>48</v>
@@ -1092,7 +1092,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://sofifa.com/team/1842/cagliari/</t>
+          <t>https://sofifa.com/team/206/hellas-verona/</t>
         </is>
       </c>
       <c r="I18" t="n">
@@ -1138,35 +1138,35 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>206</v>
+        <v>1746</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>hellas verona</t>
+          <t>empoli</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Sanderson Park</t>
+          <t>Euro Arena</t>
         </is>
       </c>
       <c r="D20" t="n">
         <v>1</v>
       </c>
       <c r="E20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F20" t="n">
-        <v>48</v>
+        <v>110374</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Napoli</t>
+          <t>Fiorentina</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>https://sofifa.com/team/206/hellas-verona/</t>
+          <t>https://sofifa.com/team/1746/empoli/</t>
         </is>
       </c>
       <c r="I20" t="n">
@@ -1207,6 +1207,746 @@
         </is>
       </c>
       <c r="I21" t="n">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="n">
+        <v>50</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>parma</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Arena d'Oro</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>3</v>
+      </c>
+      <c r="E22" t="n">
+        <v>9</v>
+      </c>
+      <c r="F22" t="n">
+        <v>189</v>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Bologna</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>https://sofifa.com/team/50/parma/</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="n">
+        <v>111434</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>cremonese</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Stadio Classico</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" t="n">
+        <v>8</v>
+      </c>
+      <c r="F23" t="n">
+        <v>1745</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Como</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>https://sofifa.com/team/111434/cremonese/</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="1" t="n">
+        <v>1745</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>como</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Town Park</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" t="n">
+        <v>5</v>
+      </c>
+      <c r="F24" t="n">
+        <v>111811</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Monza</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>https://sofifa.com/team/1745/como/</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="1" t="n">
+        <v>1837</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>sampdoria</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Stadion Europa</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E25" t="n">
+        <v>9</v>
+      </c>
+      <c r="F25" t="n">
+        <v>110556</v>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Genoa</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>https://sofifa.com/team/1837/sampdoria/</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="1" t="n">
+        <v>1843</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>palermo</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Stadio Classico</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>2</v>
+      </c>
+      <c r="E26" t="n">
+        <v>8</v>
+      </c>
+      <c r="F26" t="n">
+        <v>111657</v>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Frosinone</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>https://sofifa.com/team/1843/palermo/</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="n">
+        <v>205</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>venezia</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Town Park</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>1</v>
+      </c>
+      <c r="E27" t="n">
+        <v>7</v>
+      </c>
+      <c r="F27" t="n">
+        <v>206</v>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Hellas Verona</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>https://sofifa.com/team/205/venezia/</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="1" t="n">
+        <v>112168</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>cosenza</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Euro Arena</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>1</v>
+      </c>
+      <c r="E28" t="n">
+        <v>2</v>
+      </c>
+      <c r="F28" t="n">
+        <v>110908</v>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Catanzaro</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>https://sofifa.com/team/112168/cosenza/</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="1" t="n">
+        <v>1847</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>ascoli</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Arena d'Oro</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" t="n">
+        <v>7</v>
+      </c>
+      <c r="F29" t="n">
+        <v>206</v>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Hellas Verona</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>https://sofifa.com/team/1847/ascoli/</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="1" t="n">
+        <v>1848</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>bari 1908</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Stadion Olympik</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>2</v>
+      </c>
+      <c r="E30" t="n">
+        <v>8</v>
+      </c>
+      <c r="F30" t="n">
+        <v>347</v>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Lecce</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>https://sofifa.com/team/1848/bari-1908/</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="1" t="n">
+        <v>110908</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>catanzaro</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Stadion 23. Maj</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>1</v>
+      </c>
+      <c r="E31" t="n">
+        <v>2</v>
+      </c>
+      <c r="F31" t="n">
+        <v>112168</v>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Cosenza</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>https://sofifa.com/team/110908/catanzaro/</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="1" t="n">
+        <v>110738</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>pisa</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Stadion 23. Maj</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>1</v>
+      </c>
+      <c r="E32" t="n">
+        <v>7</v>
+      </c>
+      <c r="F32" t="n">
+        <v>110374</v>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Fiorentina</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>https://sofifa.com/team/110738/pisa/</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="1" t="n">
+        <v>110741</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>spezia</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Home stadium</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>1</v>
+      </c>
+      <c r="E33" t="n">
+        <v>8</v>
+      </c>
+      <c r="F33" t="n">
+        <v>110556</v>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Genoa</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>https://sofifa.com/team/110741/spezia/</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="1" t="n">
+        <v>112494</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>sudtirol</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Longville Stadium</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>1</v>
+      </c>
+      <c r="E34" t="n">
+        <v>4</v>
+      </c>
+      <c r="F34" t="n">
+        <v>55</v>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Udinese</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>https://sofifa.com/team/112494/sudtirol/</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="1" t="n">
+        <v>111993</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>cittadella</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Aloha Park</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>1</v>
+      </c>
+      <c r="E35" t="n">
+        <v>3</v>
+      </c>
+      <c r="F35" t="n">
+        <v>205</v>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Venezia</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>https://sofifa.com/team/111993/cittadella/</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="1" t="n">
+        <v>110740</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>reggiana</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Forest Park Stadium (Square Ground)</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>1</v>
+      </c>
+      <c r="E36" t="n">
+        <v>2</v>
+      </c>
+      <c r="F36" t="n">
+        <v>50</v>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Parma</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>https://sofifa.com/team/110740/reggiana/</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="1" t="n">
+        <v>190</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>brescia</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Home stadium</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>1</v>
+      </c>
+      <c r="E37" t="n">
+        <v>7</v>
+      </c>
+      <c r="F37" t="n">
+        <v>39</v>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Atalanta</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>https://sofifa.com/team/190/brescia/</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="1" t="n">
+        <v>1744</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>modena</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Crown Lane</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>1</v>
+      </c>
+      <c r="E38" t="n">
+        <v>5</v>
+      </c>
+      <c r="F38" t="n">
+        <v>189</v>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Bologna</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>https://sofifa.com/team/1744/modena/</t>
+        </is>
+      </c>
+      <c r="I38" t="n">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="1" t="n">
+        <v>1846</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>lecco</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Longville Stadium</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>1</v>
+      </c>
+      <c r="E39" t="n">
+        <v>1</v>
+      </c>
+      <c r="F39" t="n">
+        <v>1745</v>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Como</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>https://sofifa.com/team/1846/lecco/</t>
+        </is>
+      </c>
+      <c r="I39" t="n">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="1" t="n">
+        <v>570</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>ternana</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Stadion 23. Maj</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>1</v>
+      </c>
+      <c r="E40" t="n">
+        <v>5</v>
+      </c>
+      <c r="F40" t="n">
+        <v>1847</v>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Ascoli</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>https://sofifa.com/team/570/ternana/</t>
+        </is>
+      </c>
+      <c r="I40" t="n">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="1" t="n">
+        <v>112499</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>feralpisalò</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Euro Arena</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>1</v>
+      </c>
+      <c r="E41" t="n">
+        <v>2</v>
+      </c>
+      <c r="F41" t="n">
+        <v>111434</v>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Cremonese</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>https://sofifa.com/team/112499/feralpisalo/</t>
+        </is>
+      </c>
+      <c r="I41" t="n">
         <v>77</v>
       </c>
     </row>

</xml_diff>